<commit_message>
privacy: strip personal metadata and machine paths from committed artifacts
- crm-shadow-pilot-result.xlsx: remove the xl/persons/person.xml threaded-comment
  person part and its content-type/relationship entries. The author display name
  leaked a real personal name in hidden package metadata; workbook cell content is
  byte-identical (7 sheets, 954 cells) and the deliberate owner attribution cell is
  untouched.
- local-release-check.json (both packages): replace machine-specific absolute roots
  with the machine-independent package name. JSON structure, gates and summary are
  unchanged.
</commit_message>
<xml_diff>
--- a/outputs/crm-shadow-pilot-20260816/crm-shadow-pilot-result.xlsx
+++ b/outputs/crm-shadow-pilot-20260816/crm-shadow-pilot-result.xlsx
@@ -400,12 +400,6 @@
 </x:styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Kang Jiaxin" id="{5B6826FB-0F7B-4CDC-9F15-DF0007406F74}"/>
-</xltc:personList>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
   <a:themeElements>

</xml_diff>